<commit_message>
Make the tracking sheet import-ready for Pathment
Added an Email key column to the Mentee Tracker, mentee-name dropdowns on the Daily Log and 1-on-1 Log sourced from the tracker so names always match, and import-format.md documenting exactly how each tab and column maps to Pathment (with allowed values). The goal is that filling the sheet normally now means it can import straight into Pathment later, without any extra work.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mentor-tracking-sheet/Dev Weekend - Mentee Tracker.xlsx
+++ b/mentor-tracking-sheet/Dev Weekend - Mentee Tracker.xlsx
@@ -48,13 +48,13 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="001F2933"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="001F2933"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -106,12 +106,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -527,11 +527,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="88" customWidth="1" min="2" max="2"/>
+    <col width="92" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -549,255 +549,275 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
-      <c r="B4" s="3" t="inlineStr"/>
+      <c r="A4" s="3" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>How to use</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr"/>
+      <c r="B5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Open in Google Sheets (File, Import, Upload) or Excel. Share with your co-mentors.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Mentee Tracker is the main view. One row per mentee, one glance at where everyone is.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Daily Log is the day-by-day habit and task tracking. Add a row per mentee per day.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>4.</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>1-on-1 Log is for sessions. Every note records who logged it, so attribution stays clear.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>5.</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Keep it honest. The sheet is to help people, not to grade them.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
-      <c r="B11" s="3" t="inlineStr"/>
+      <c r="A11" s="3" t="inlineStr"/>
+      <c r="B11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Built to import into Pathment later</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr"/>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Keep the header rows and the dropdown values as they are, and one mentee per row, and Pathment will be able to import this sheet straight in when it is ready. Email is the key that links a mentee across tabs. See import-format.md for the details. You do not need to do anything extra, just fill the sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>What the columns mean</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>The mentee's email. The unique key that ties their rows together across tabs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Absolute %</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Raw output against the plan. Honest and unforgiving.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Relative %</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Progress given the circumstances the mentee has logged. The fair read of effort.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>On-time %</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Share of work submitted by its date.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Momentum</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Up, Flat, or Down over recent weeks.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Sentiment</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Positive, Neutral, or Low. The engagement and mood read.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>On track, Watch, or At risk. Colour-coded so the people who need you stand out.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Consistency / Communication / Resilience / Independence</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>The working-style read, 0 to 100. A gentle read of how someone works, not a grade.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
-      <c r="B20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>This sheet follows the Dev Weekend methodology. Pathment will automate it later.</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>At a glance (updates from the tracker)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Mentees tracked</t>
         </is>
       </c>
-      <c r="B24" s="6">
+      <c r="B26" s="6">
         <f>COUNTA('Mentee Tracker'!A2:A200)</f>
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>On track</t>
         </is>
       </c>
-      <c r="B25" s="6">
-        <f>COUNTIF('Mentee Tracker'!M2:M200,"On track")</f>
+      <c r="B27" s="6">
+        <f>COUNTIF('Mentee Tracker'!N2:N200,"On track")</f>
         <v/>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Watch</t>
         </is>
       </c>
-      <c r="B26" s="6">
-        <f>COUNTIF('Mentee Tracker'!M2:M200,"Watch")</f>
+      <c r="B28" s="6">
+        <f>COUNTIF('Mentee Tracker'!N2:N200,"Watch")</f>
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>At risk</t>
         </is>
       </c>
-      <c r="B27" s="6">
-        <f>COUNTIF('Mentee Tracker'!M2:M200,"At risk")</f>
+      <c r="B29" s="6">
+        <f>COUNTIF('Mentee Tracker'!N2:N200,"At risk")</f>
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>Average on-time %</t>
         </is>
       </c>
-      <c r="B28" s="6">
-        <f>IFERROR(ROUND(AVERAGE('Mentee Tracker'!J2:J200),0),0)</f>
+      <c r="B30" s="6">
+        <f>IFERROR(ROUND(AVERAGE('Mentee Tracker'!K2:K200),0),0)</f>
         <v/>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Average absolute %</t>
         </is>
       </c>
-      <c r="B29" s="6">
-        <f>IFERROR(ROUND(AVERAGE('Mentee Tracker'!H2:H200),0),0)</f>
+      <c r="B31" s="6">
+        <f>IFERROR(ROUND(AVERAGE('Mentee Tracker'!I2:I200),0),0)</f>
         <v/>
       </c>
     </row>
@@ -812,32 +832,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W19"/>
+  <dimension ref="A1:X19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="9" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
-    <col width="13" customWidth="1" min="20" max="20"/>
-    <col width="10" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="52" customWidth="1" min="23" max="23"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="52" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -848,110 +869,115 @@
       </c>
       <c r="B1" s="7" t="inlineStr">
         <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
           <t>Clan</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Current roadmap</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>Current step</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>Absolute %</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>Relative %</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>On-time %</t>
         </is>
       </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="L1" s="7" t="inlineStr">
         <is>
           <t>Momentum</t>
         </is>
       </c>
-      <c r="L1" s="7" t="inlineStr">
+      <c r="M1" s="7" t="inlineStr">
         <is>
           <t>Sentiment</t>
         </is>
       </c>
-      <c r="M1" s="7" t="inlineStr">
+      <c r="N1" s="7" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
       </c>
-      <c r="N1" s="7" t="inlineStr">
+      <c r="O1" s="7" t="inlineStr">
         <is>
           <t>Open blockers</t>
         </is>
       </c>
-      <c r="O1" s="7" t="inlineStr">
+      <c r="P1" s="7" t="inlineStr">
         <is>
           <t>Last active</t>
         </is>
       </c>
-      <c r="P1" s="7" t="inlineStr">
+      <c r="Q1" s="7" t="inlineStr">
         <is>
           <t>Nudges (wk)</t>
         </is>
       </c>
-      <c r="Q1" s="7" t="inlineStr">
+      <c r="R1" s="7" t="inlineStr">
         <is>
           <t>Last 1:1</t>
         </is>
       </c>
-      <c r="R1" s="7" t="inlineStr">
+      <c r="S1" s="7" t="inlineStr">
         <is>
           <t>Next 1:1</t>
         </is>
       </c>
-      <c r="S1" s="7" t="inlineStr">
+      <c r="T1" s="7" t="inlineStr">
         <is>
           <t>Consistency</t>
         </is>
       </c>
-      <c r="T1" s="7" t="inlineStr">
+      <c r="U1" s="7" t="inlineStr">
         <is>
           <t>Communication</t>
         </is>
       </c>
-      <c r="U1" s="7" t="inlineStr">
+      <c r="V1" s="7" t="inlineStr">
         <is>
           <t>Resilience</t>
         </is>
       </c>
-      <c r="V1" s="7" t="inlineStr">
+      <c r="W1" s="7" t="inlineStr">
         <is>
           <t>Independence</t>
         </is>
       </c>
-      <c r="W1" s="7" t="inlineStr">
+      <c r="X1" s="7" t="inlineStr">
         <is>
           <t>Mentor notes / next steps</t>
         </is>
@@ -965,92 +991,97 @@
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
+          <t>aisha.k@email.com</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
           <t>Phoenix Clan</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>Intermediate</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>Toronto, CA</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>6/12</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>Backend Foundations</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>3. Add authentication</t>
         </is>
       </c>
-      <c r="H2" s="9" t="n">
+      <c r="I2" s="9" t="n">
         <v>72</v>
       </c>
-      <c r="I2" s="9" t="n">
+      <c r="J2" s="9" t="n">
         <v>88</v>
       </c>
-      <c r="J2" s="9" t="n">
+      <c r="K2" s="9" t="n">
         <v>84</v>
       </c>
-      <c r="K2" s="9" t="inlineStr">
+      <c r="L2" s="9" t="inlineStr">
         <is>
           <t>Up</t>
         </is>
       </c>
-      <c r="L2" s="9" t="inlineStr">
+      <c r="M2" s="9" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="M2" s="9" t="inlineStr">
+      <c r="N2" s="9" t="inlineStr">
         <is>
           <t>On track</t>
         </is>
       </c>
-      <c r="N2" s="9" t="n">
+      <c r="O2" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="O2" s="9" t="inlineStr">
+      <c r="P2" s="9" t="inlineStr">
         <is>
           <t>2h ago</t>
         </is>
       </c>
-      <c r="P2" s="9" t="n">
+      <c r="Q2" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Q2" s="9" t="inlineStr">
+      <c r="R2" s="9" t="inlineStr">
         <is>
           <t>May 15</t>
         </is>
       </c>
-      <c r="R2" s="9" t="inlineStr">
+      <c r="S2" s="9" t="inlineStr">
         <is>
           <t>Thu, May 29</t>
         </is>
       </c>
-      <c r="S2" s="9" t="n">
+      <c r="T2" s="9" t="n">
         <v>85</v>
       </c>
-      <c r="T2" s="9" t="n">
+      <c r="U2" s="9" t="n">
         <v>78</v>
       </c>
-      <c r="U2" s="9" t="n">
+      <c r="V2" s="9" t="n">
         <v>92</v>
       </c>
-      <c r="V2" s="9" t="n">
+      <c r="W2" s="9" t="n">
         <v>70</v>
       </c>
-      <c r="W2" s="10" t="inlineStr">
+      <c r="X2" s="10" t="inlineStr">
         <is>
           <t>Two submissions waiting. JWT refresh-token blocker flagged early. Pair on auth Thursday.</t>
         </is>
@@ -1064,92 +1095,97 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
+          <t>diego.m@email.com</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
           <t>Phoenix Clan</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Intermediate</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>Lahore, PK</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>6/12</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>Frontend Craft</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="H3" s="8" t="inlineStr">
         <is>
           <t>1. Component composition</t>
         </is>
       </c>
-      <c r="H3" s="9" t="n">
+      <c r="I3" s="9" t="n">
         <v>41</v>
       </c>
-      <c r="I3" s="9" t="n">
+      <c r="J3" s="9" t="n">
         <v>79</v>
       </c>
-      <c r="J3" s="9" t="n">
+      <c r="K3" s="9" t="n">
         <v>58</v>
       </c>
-      <c r="K3" s="9" t="inlineStr">
+      <c r="L3" s="9" t="inlineStr">
         <is>
           <t>Up</t>
         </is>
       </c>
-      <c r="L3" s="9" t="inlineStr">
+      <c r="M3" s="9" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="M3" s="9" t="inlineStr">
+      <c r="N3" s="9" t="inlineStr">
         <is>
           <t>Watch</t>
         </is>
       </c>
-      <c r="N3" s="9" t="n">
+      <c r="O3" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="O3" s="9" t="inlineStr">
+      <c r="P3" s="9" t="inlineStr">
         <is>
           <t>1d ago</t>
         </is>
       </c>
-      <c r="P3" s="9" t="n">
+      <c r="Q3" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Q3" s="9" t="inlineStr">
+      <c r="R3" s="9" t="inlineStr">
         <is>
           <t>May 18</t>
         </is>
       </c>
-      <c r="R3" s="9" t="inlineStr">
+      <c r="S3" s="9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="S3" s="9" t="n">
+      <c r="T3" s="9" t="n">
         <v>55</v>
       </c>
-      <c r="T3" s="9" t="n">
+      <c r="U3" s="9" t="n">
         <v>72</v>
       </c>
-      <c r="U3" s="9" t="n">
+      <c r="V3" s="9" t="n">
         <v>95</v>
       </c>
-      <c r="V3" s="9" t="n">
+      <c r="W3" s="9" t="n">
         <v>60</v>
       </c>
-      <c r="W3" s="10" t="inlineStr">
+      <c r="X3" s="10" t="inlineStr">
         <is>
           <t>Power outages and a shared machine. Struggling despite effort. Protect deadlines, shift due times to AM PKT.</t>
         </is>
@@ -1163,92 +1199,97 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
+          <t>priya.n@email.com</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
           <t>Phoenix Clan</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>Intermediate</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>Bengaluru, IN</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>6/12</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H4" s="9" t="n">
+      <c r="I4" s="9" t="n">
         <v>31</v>
       </c>
-      <c r="I4" s="9" t="n">
+      <c r="J4" s="9" t="n">
         <v>34</v>
       </c>
-      <c r="J4" s="9" t="n">
+      <c r="K4" s="9" t="n">
         <v>44</v>
       </c>
-      <c r="K4" s="9" t="inlineStr">
+      <c r="L4" s="9" t="inlineStr">
         <is>
           <t>Down</t>
         </is>
       </c>
-      <c r="L4" s="9" t="inlineStr">
+      <c r="M4" s="9" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="M4" s="9" t="inlineStr">
+      <c r="N4" s="9" t="inlineStr">
         <is>
           <t>At risk</t>
         </is>
       </c>
-      <c r="N4" s="9" t="n">
+      <c r="O4" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="O4" s="9" t="inlineStr">
+      <c r="P4" s="9" t="inlineStr">
         <is>
           <t>6d ago</t>
         </is>
       </c>
-      <c r="P4" s="9" t="n">
+      <c r="Q4" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="Q4" s="9" t="inlineStr">
+      <c r="R4" s="9" t="inlineStr">
         <is>
           <t>May 20</t>
         </is>
       </c>
-      <c r="R4" s="9" t="inlineStr">
+      <c r="S4" s="9" t="inlineStr">
         <is>
           <t>Wed, May 28</t>
         </is>
       </c>
-      <c r="S4" s="9" t="n">
+      <c r="T4" s="9" t="n">
         <v>40</v>
       </c>
-      <c r="T4" s="9" t="n">
+      <c r="U4" s="9" t="n">
         <v>38</v>
       </c>
-      <c r="U4" s="9" t="n">
+      <c r="V4" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="V4" s="9" t="n">
+      <c r="W4" s="9" t="n">
         <v>65</v>
       </c>
-      <c r="W4" s="10" t="inlineStr">
+      <c r="X4" s="10" t="inlineStr">
         <is>
           <t>Disengagement risk. No login for 6 days, two nudges unanswered. Direct warm check-in. Psychologist session held May 20.</t>
         </is>
@@ -1262,92 +1303,97 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
+          <t>liam.w@email.com</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
           <t>Phoenix Clan</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Intermediate</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Dublin, IE</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>6/12</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H5" s="9" t="n">
+      <c r="I5" s="9" t="n">
         <v>95</v>
       </c>
-      <c r="I5" s="9" t="n">
+      <c r="J5" s="9" t="n">
         <v>76</v>
       </c>
-      <c r="J5" s="9" t="n">
+      <c r="K5" s="9" t="n">
         <v>97</v>
       </c>
-      <c r="K5" s="9" t="inlineStr">
+      <c r="L5" s="9" t="inlineStr">
         <is>
           <t>Flat</t>
         </is>
       </c>
-      <c r="L5" s="9" t="inlineStr">
+      <c r="M5" s="9" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="M5" s="9" t="inlineStr">
+      <c r="N5" s="9" t="inlineStr">
         <is>
           <t>On track</t>
         </is>
       </c>
-      <c r="N5" s="9" t="n">
+      <c r="O5" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="O5" s="9" t="inlineStr">
+      <c r="P5" s="9" t="inlineStr">
         <is>
           <t>5h ago</t>
         </is>
       </c>
-      <c r="P5" s="9" t="n">
+      <c r="Q5" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Q5" s="9" t="inlineStr">
+      <c r="R5" s="9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="R5" s="9" t="inlineStr">
+      <c r="S5" s="9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="S5" s="9" t="n">
+      <c r="T5" s="9" t="n">
         <v>96</v>
       </c>
-      <c r="T5" s="9" t="n">
+      <c r="U5" s="9" t="n">
         <v>65</v>
       </c>
-      <c r="U5" s="9" t="n">
+      <c r="V5" s="9" t="n">
         <v>70</v>
       </c>
-      <c r="V5" s="9" t="n">
+      <c r="W5" s="9" t="n">
         <v>90</v>
       </c>
-      <c r="W5" s="10" t="inlineStr">
+      <c r="X5" s="10" t="inlineStr">
         <is>
           <t>Top of cohort on output, almost always early. May be coasting on easy ground. Add a stretch track.</t>
         </is>
@@ -1361,92 +1407,97 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
+          <t>fatima.n@email.com</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
           <t>Phoenix Clan</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>Intermediate</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>Karachi, PK</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>6/12</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="G6" s="8" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="H6" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H6" s="9" t="n">
+      <c r="I6" s="9" t="n">
         <v>64</v>
       </c>
-      <c r="I6" s="9" t="n">
+      <c r="J6" s="9" t="n">
         <v>71</v>
       </c>
-      <c r="J6" s="9" t="n">
+      <c r="K6" s="9" t="n">
         <v>79</v>
       </c>
-      <c r="K6" s="9" t="inlineStr">
+      <c r="L6" s="9" t="inlineStr">
         <is>
           <t>Up</t>
         </is>
       </c>
-      <c r="L6" s="9" t="inlineStr">
+      <c r="M6" s="9" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="M6" s="9" t="inlineStr">
+      <c r="N6" s="9" t="inlineStr">
         <is>
           <t>On track</t>
         </is>
       </c>
-      <c r="N6" s="9" t="n">
+      <c r="O6" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="O6" s="9" t="inlineStr">
+      <c r="P6" s="9" t="inlineStr">
         <is>
           <t>3h ago</t>
         </is>
       </c>
-      <c r="P6" s="9" t="n">
+      <c r="Q6" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Q6" s="9" t="inlineStr">
+      <c r="R6" s="9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="R6" s="9" t="inlineStr">
+      <c r="S6" s="9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="S6" s="9" t="n">
+      <c r="T6" s="9" t="n">
         <v>80</v>
       </c>
-      <c r="T6" s="9" t="n">
+      <c r="U6" s="9" t="n">
         <v>85</v>
       </c>
-      <c r="U6" s="9" t="n">
+      <c r="V6" s="9" t="n">
         <v>75</v>
       </c>
-      <c r="V6" s="9" t="n">
+      <c r="W6" s="9" t="n">
         <v>72</v>
       </c>
-      <c r="W6" s="10" t="inlineStr">
+      <c r="X6" s="10" t="inlineStr">
         <is>
           <t>Solid and improving three weeks running. One async/await blocker, working at it.</t>
         </is>
@@ -1460,92 +1511,97 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
+          <t>tomas.b@email.com</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
           <t>Phoenix Clan</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>Intermediate</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Oslo, NO</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>6/12</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="H7" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H7" s="9" t="n">
+      <c r="I7" s="9" t="n">
         <v>53</v>
       </c>
-      <c r="I7" s="9" t="n">
+      <c r="J7" s="9" t="n">
         <v>49</v>
       </c>
-      <c r="J7" s="9" t="n">
+      <c r="K7" s="9" t="n">
         <v>62</v>
       </c>
-      <c r="K7" s="9" t="inlineStr">
+      <c r="L7" s="9" t="inlineStr">
         <is>
           <t>Down</t>
         </is>
       </c>
-      <c r="L7" s="9" t="inlineStr">
+      <c r="M7" s="9" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="M7" s="9" t="inlineStr">
+      <c r="N7" s="9" t="inlineStr">
         <is>
           <t>Watch</t>
         </is>
       </c>
-      <c r="N7" s="9" t="n">
+      <c r="O7" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="O7" s="9" t="inlineStr">
+      <c r="P7" s="9" t="inlineStr">
         <is>
           <t>2d ago</t>
         </is>
       </c>
-      <c r="P7" s="9" t="n">
+      <c r="Q7" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Q7" s="9" t="inlineStr">
+      <c r="R7" s="9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="R7" s="9" t="inlineStr">
+      <c r="S7" s="9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="S7" s="9" t="n">
+      <c r="T7" s="9" t="n">
         <v>60</v>
       </c>
-      <c r="T7" s="9" t="n">
+      <c r="U7" s="9" t="n">
         <v>70</v>
       </c>
-      <c r="U7" s="9" t="n">
+      <c r="V7" s="9" t="n">
         <v>64</v>
       </c>
-      <c r="V7" s="9" t="n">
+      <c r="W7" s="9" t="n">
         <v>68</v>
       </c>
-      <c r="W7" s="10" t="inlineStr">
+      <c r="X7" s="10" t="inlineStr">
         <is>
           <t>Drifting, two late tasks this week. Still responsive. A short check-in now prevents a bigger slide.</t>
         </is>
@@ -1559,7 +1615,7 @@
       <c r="E8" s="8" t="inlineStr"/>
       <c r="F8" s="8" t="inlineStr"/>
       <c r="G8" s="8" t="inlineStr"/>
-      <c r="H8" s="9" t="inlineStr"/>
+      <c r="H8" s="8" t="inlineStr"/>
       <c r="I8" s="9" t="inlineStr"/>
       <c r="J8" s="9" t="inlineStr"/>
       <c r="K8" s="9" t="inlineStr"/>
@@ -1574,7 +1630,8 @@
       <c r="T8" s="9" t="inlineStr"/>
       <c r="U8" s="9" t="inlineStr"/>
       <c r="V8" s="9" t="inlineStr"/>
-      <c r="W8" s="10" t="inlineStr"/>
+      <c r="W8" s="9" t="inlineStr"/>
+      <c r="X8" s="10" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr"/>
@@ -1584,7 +1641,7 @@
       <c r="E9" s="8" t="inlineStr"/>
       <c r="F9" s="8" t="inlineStr"/>
       <c r="G9" s="8" t="inlineStr"/>
-      <c r="H9" s="9" t="inlineStr"/>
+      <c r="H9" s="8" t="inlineStr"/>
       <c r="I9" s="9" t="inlineStr"/>
       <c r="J9" s="9" t="inlineStr"/>
       <c r="K9" s="9" t="inlineStr"/>
@@ -1599,7 +1656,8 @@
       <c r="T9" s="9" t="inlineStr"/>
       <c r="U9" s="9" t="inlineStr"/>
       <c r="V9" s="9" t="inlineStr"/>
-      <c r="W9" s="10" t="inlineStr"/>
+      <c r="W9" s="9" t="inlineStr"/>
+      <c r="X9" s="10" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr"/>
@@ -1609,7 +1667,7 @@
       <c r="E10" s="8" t="inlineStr"/>
       <c r="F10" s="8" t="inlineStr"/>
       <c r="G10" s="8" t="inlineStr"/>
-      <c r="H10" s="9" t="inlineStr"/>
+      <c r="H10" s="8" t="inlineStr"/>
       <c r="I10" s="9" t="inlineStr"/>
       <c r="J10" s="9" t="inlineStr"/>
       <c r="K10" s="9" t="inlineStr"/>
@@ -1624,7 +1682,8 @@
       <c r="T10" s="9" t="inlineStr"/>
       <c r="U10" s="9" t="inlineStr"/>
       <c r="V10" s="9" t="inlineStr"/>
-      <c r="W10" s="10" t="inlineStr"/>
+      <c r="W10" s="9" t="inlineStr"/>
+      <c r="X10" s="10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr"/>
@@ -1634,7 +1693,7 @@
       <c r="E11" s="8" t="inlineStr"/>
       <c r="F11" s="8" t="inlineStr"/>
       <c r="G11" s="8" t="inlineStr"/>
-      <c r="H11" s="9" t="inlineStr"/>
+      <c r="H11" s="8" t="inlineStr"/>
       <c r="I11" s="9" t="inlineStr"/>
       <c r="J11" s="9" t="inlineStr"/>
       <c r="K11" s="9" t="inlineStr"/>
@@ -1649,7 +1708,8 @@
       <c r="T11" s="9" t="inlineStr"/>
       <c r="U11" s="9" t="inlineStr"/>
       <c r="V11" s="9" t="inlineStr"/>
-      <c r="W11" s="10" t="inlineStr"/>
+      <c r="W11" s="9" t="inlineStr"/>
+      <c r="X11" s="10" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr"/>
@@ -1659,7 +1719,7 @@
       <c r="E12" s="8" t="inlineStr"/>
       <c r="F12" s="8" t="inlineStr"/>
       <c r="G12" s="8" t="inlineStr"/>
-      <c r="H12" s="9" t="inlineStr"/>
+      <c r="H12" s="8" t="inlineStr"/>
       <c r="I12" s="9" t="inlineStr"/>
       <c r="J12" s="9" t="inlineStr"/>
       <c r="K12" s="9" t="inlineStr"/>
@@ -1674,7 +1734,8 @@
       <c r="T12" s="9" t="inlineStr"/>
       <c r="U12" s="9" t="inlineStr"/>
       <c r="V12" s="9" t="inlineStr"/>
-      <c r="W12" s="10" t="inlineStr"/>
+      <c r="W12" s="9" t="inlineStr"/>
+      <c r="X12" s="10" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr"/>
@@ -1684,7 +1745,7 @@
       <c r="E13" s="8" t="inlineStr"/>
       <c r="F13" s="8" t="inlineStr"/>
       <c r="G13" s="8" t="inlineStr"/>
-      <c r="H13" s="9" t="inlineStr"/>
+      <c r="H13" s="8" t="inlineStr"/>
       <c r="I13" s="9" t="inlineStr"/>
       <c r="J13" s="9" t="inlineStr"/>
       <c r="K13" s="9" t="inlineStr"/>
@@ -1699,7 +1760,8 @@
       <c r="T13" s="9" t="inlineStr"/>
       <c r="U13" s="9" t="inlineStr"/>
       <c r="V13" s="9" t="inlineStr"/>
-      <c r="W13" s="10" t="inlineStr"/>
+      <c r="W13" s="9" t="inlineStr"/>
+      <c r="X13" s="10" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr"/>
@@ -1709,7 +1771,7 @@
       <c r="E14" s="8" t="inlineStr"/>
       <c r="F14" s="8" t="inlineStr"/>
       <c r="G14" s="8" t="inlineStr"/>
-      <c r="H14" s="9" t="inlineStr"/>
+      <c r="H14" s="8" t="inlineStr"/>
       <c r="I14" s="9" t="inlineStr"/>
       <c r="J14" s="9" t="inlineStr"/>
       <c r="K14" s="9" t="inlineStr"/>
@@ -1724,7 +1786,8 @@
       <c r="T14" s="9" t="inlineStr"/>
       <c r="U14" s="9" t="inlineStr"/>
       <c r="V14" s="9" t="inlineStr"/>
-      <c r="W14" s="10" t="inlineStr"/>
+      <c r="W14" s="9" t="inlineStr"/>
+      <c r="X14" s="10" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr"/>
@@ -1734,7 +1797,7 @@
       <c r="E15" s="8" t="inlineStr"/>
       <c r="F15" s="8" t="inlineStr"/>
       <c r="G15" s="8" t="inlineStr"/>
-      <c r="H15" s="9" t="inlineStr"/>
+      <c r="H15" s="8" t="inlineStr"/>
       <c r="I15" s="9" t="inlineStr"/>
       <c r="J15" s="9" t="inlineStr"/>
       <c r="K15" s="9" t="inlineStr"/>
@@ -1749,7 +1812,8 @@
       <c r="T15" s="9" t="inlineStr"/>
       <c r="U15" s="9" t="inlineStr"/>
       <c r="V15" s="9" t="inlineStr"/>
-      <c r="W15" s="10" t="inlineStr"/>
+      <c r="W15" s="9" t="inlineStr"/>
+      <c r="X15" s="10" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr"/>
@@ -1759,7 +1823,7 @@
       <c r="E16" s="8" t="inlineStr"/>
       <c r="F16" s="8" t="inlineStr"/>
       <c r="G16" s="8" t="inlineStr"/>
-      <c r="H16" s="9" t="inlineStr"/>
+      <c r="H16" s="8" t="inlineStr"/>
       <c r="I16" s="9" t="inlineStr"/>
       <c r="J16" s="9" t="inlineStr"/>
       <c r="K16" s="9" t="inlineStr"/>
@@ -1774,7 +1838,8 @@
       <c r="T16" s="9" t="inlineStr"/>
       <c r="U16" s="9" t="inlineStr"/>
       <c r="V16" s="9" t="inlineStr"/>
-      <c r="W16" s="10" t="inlineStr"/>
+      <c r="W16" s="9" t="inlineStr"/>
+      <c r="X16" s="10" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr"/>
@@ -1784,7 +1849,7 @@
       <c r="E17" s="8" t="inlineStr"/>
       <c r="F17" s="8" t="inlineStr"/>
       <c r="G17" s="8" t="inlineStr"/>
-      <c r="H17" s="9" t="inlineStr"/>
+      <c r="H17" s="8" t="inlineStr"/>
       <c r="I17" s="9" t="inlineStr"/>
       <c r="J17" s="9" t="inlineStr"/>
       <c r="K17" s="9" t="inlineStr"/>
@@ -1799,7 +1864,8 @@
       <c r="T17" s="9" t="inlineStr"/>
       <c r="U17" s="9" t="inlineStr"/>
       <c r="V17" s="9" t="inlineStr"/>
-      <c r="W17" s="10" t="inlineStr"/>
+      <c r="W17" s="9" t="inlineStr"/>
+      <c r="X17" s="10" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr"/>
@@ -1809,7 +1875,7 @@
       <c r="E18" s="8" t="inlineStr"/>
       <c r="F18" s="8" t="inlineStr"/>
       <c r="G18" s="8" t="inlineStr"/>
-      <c r="H18" s="9" t="inlineStr"/>
+      <c r="H18" s="8" t="inlineStr"/>
       <c r="I18" s="9" t="inlineStr"/>
       <c r="J18" s="9" t="inlineStr"/>
       <c r="K18" s="9" t="inlineStr"/>
@@ -1824,7 +1890,8 @@
       <c r="T18" s="9" t="inlineStr"/>
       <c r="U18" s="9" t="inlineStr"/>
       <c r="V18" s="9" t="inlineStr"/>
-      <c r="W18" s="10" t="inlineStr"/>
+      <c r="W18" s="9" t="inlineStr"/>
+      <c r="X18" s="10" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr"/>
@@ -1834,7 +1901,7 @@
       <c r="E19" s="8" t="inlineStr"/>
       <c r="F19" s="8" t="inlineStr"/>
       <c r="G19" s="8" t="inlineStr"/>
-      <c r="H19" s="9" t="inlineStr"/>
+      <c r="H19" s="8" t="inlineStr"/>
       <c r="I19" s="9" t="inlineStr"/>
       <c r="J19" s="9" t="inlineStr"/>
       <c r="K19" s="9" t="inlineStr"/>
@@ -1849,10 +1916,11 @@
       <c r="T19" s="9" t="inlineStr"/>
       <c r="U19" s="9" t="inlineStr"/>
       <c r="V19" s="9" t="inlineStr"/>
-      <c r="W19" s="10" t="inlineStr"/>
+      <c r="W19" s="9" t="inlineStr"/>
+      <c r="X19" s="10" t="inlineStr"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="M2:M19">
+  <conditionalFormatting sqref="N2:N19">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"At risk"</formula>
     </cfRule>
@@ -1864,13 +1932,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="K2:K19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Up,Flat,Down"</formula1>
     </dataValidation>
-    <dataValidation sqref="L2:L19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Positive,Neutral,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"On track,Watch,At risk"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2546,9 +2614,12 @@
       <c r="L26" s="10" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="C2:J26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,-"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B2:B26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'Mentee Tracker'!$A$2:$A$50</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2981,13 +3052,16 @@
       <c r="H25" s="10" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="D2:D25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"1:1,Pairing session,Career chat,Psychological session,Check-in"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Positive,Neutral,Low"</formula1>
     </dataValidation>
+    <dataValidation sqref="B2:B25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'Mentee Tracker'!$A$2:$A$50</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Make the Weekly Tracker a marking sheet: tasks discussed, done, points
The Weekly Tracker is what the mentor fills each week. Reworked its columns around marking against the tasks discussed: Tasks discussed, Tasks done, Done %, Points out of 10, Risk, and a feedback note, with the present check kept. Added a Points to date column on the Mentee Tracker that sums each mentee's weekly points by email. Week one is prefilled as a worked example. Updated import-format.md and the README.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mentor-tracking-sheet/Dev Weekend - Mentee Tracker.xlsx
+++ b/mentor-tracking-sheet/Dev Weekend - Mentee Tracker.xlsx
@@ -117,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -144,6 +144,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -548,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -601,7 +604,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Weekly Tracker is the main view. Every week has a blue bar with its date, and all mentees are already listed under it. Fill in their row for the week.</t>
+          <t>Weekly Tracker is what you fill each week. Every week has a dated bar with all mentees under it. For each mentee write the tasks you discussed, mark how much they did, and give points out of 10.</t>
         </is>
       </c>
     </row>
@@ -613,7 +616,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Mentee Tracker is the current snapshot, one row per mentee.</t>
+          <t>Mentee Tracker is the current snapshot, one row per mentee, with their points to date.</t>
         </is>
       </c>
     </row>
@@ -657,7 +660,7 @@
       <c r="A13" s="3" t="inlineStr"/>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Each blue bar is a new week, dated. Under it the same mentees are copied in as ready placeholders, so you just fill the week. Weeks are laid out ahead of time, copy the last block to add more.</t>
+          <t>Each blue bar is a new week, dated. Under it the same mentees are copied in as ready rows, so you just fill the week. Weeks are laid out ahead, copy the last block to add more.</t>
         </is>
       </c>
     </row>
@@ -696,121 +699,133 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Absolute %</t>
+          <t>Tasks discussed</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Raw output against the plan. Honest and unforgiving.</t>
+          <t>What you agreed the mentee would do this week.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Relative %</t>
+          <t>Tasks done</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Progress given the circumstances the mentee has logged. The fair read of effort.</t>
+          <t>What they actually got through.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Risk</t>
+          <t>Done %</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>On track, Watch, or At risk. Colour-coded so the people who need you stand out.</t>
+          <t>How much of the discussed tasks they completed, 0 to 100.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Consistency / Communication / Resilience / Independence</t>
+          <t>Points (/10)</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>The working-style read, 0 to 100. A gentle read, not a grade.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+          <t>Your mark for the week against what was discussed. Effort and outcome together.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>On track, Watch, or At risk. Colour-coded so the people who need you stand out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>At a glance (updates from the tracker)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Mentees tracked</t>
         </is>
       </c>
-      <c r="B25" s="6">
+      <c r="B26" s="6">
         <f>COUNTA('Mentee Tracker'!A2:A200)</f>
         <v/>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>On track</t>
         </is>
       </c>
-      <c r="B26" s="6">
+      <c r="B27" s="6">
         <f>COUNTIF('Mentee Tracker'!N2:N200,"On track")</f>
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Watch</t>
         </is>
       </c>
-      <c r="B27" s="6">
+      <c r="B28" s="6">
         <f>COUNTIF('Mentee Tracker'!N2:N200,"Watch")</f>
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>At risk</t>
         </is>
       </c>
-      <c r="B28" s="6">
+      <c r="B29" s="6">
         <f>COUNTIF('Mentee Tracker'!N2:N200,"At risk")</f>
         <v/>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>Average on-time %</t>
         </is>
       </c>
-      <c r="B29" s="6">
+      <c r="B30" s="6">
         <f>IFERROR(ROUND(AVERAGE('Mentee Tracker'!K2:K200),0),0)</f>
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>Average absolute %</t>
-        </is>
-      </c>
-      <c r="B30" s="6">
-        <f>IFERROR(ROUND(AVERAGE('Mentee Tracker'!I2:I200),0),0)</f>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Average points (latest week)</t>
+        </is>
+      </c>
+      <c r="B31" s="6">
+        <f>IFERROR(ROUND(AVERAGEIF('Weekly Tracker'!H2:H1000,"&gt;0"),1),0)</f>
         <v/>
       </c>
     </row>
@@ -825,22 +840,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M85"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="46" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -866,47 +878,32 @@
       </c>
       <c r="E1" s="7" t="inlineStr">
         <is>
-          <t>Absolute %</t>
+          <t>Tasks discussed</t>
         </is>
       </c>
       <c r="F1" s="7" t="inlineStr">
         <is>
-          <t>Relative %</t>
+          <t>Tasks done</t>
         </is>
       </c>
       <c r="G1" s="7" t="inlineStr">
         <is>
-          <t>On-time %</t>
+          <t>Done %</t>
         </is>
       </c>
       <c r="H1" s="7" t="inlineStr">
         <is>
-          <t>Momentum</t>
+          <t>Points (/10)</t>
         </is>
       </c>
       <c r="I1" s="7" t="inlineStr">
         <is>
-          <t>Sentiment</t>
+          <t>Risk</t>
         </is>
       </c>
       <c r="J1" s="7" t="inlineStr">
         <is>
-          <t>Risk</t>
-        </is>
-      </c>
-      <c r="K1" s="7" t="inlineStr">
-        <is>
-          <t>Open blockers</t>
-        </is>
-      </c>
-      <c r="L1" s="7" t="inlineStr">
-        <is>
-          <t>1:1 this week</t>
-        </is>
-      </c>
-      <c r="M1" s="7" t="inlineStr">
-        <is>
-          <t>Note / focus for next week</t>
+          <t>Feedback / focus for next week</t>
         </is>
       </c>
     </row>
@@ -936,41 +933,30 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E3" s="11" t="n">
-        <v>72</v>
-      </c>
-      <c r="F3" s="11" t="n">
-        <v>88</v>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>Finish CRUD API, start auth (JWT)</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>CRUD API done, auth started</t>
+        </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>84</v>
-      </c>
-      <c r="H3" s="11" t="inlineStr">
-        <is>
-          <t>Up</t>
-        </is>
+        <v>80</v>
+      </c>
+      <c r="H3" s="11" t="n">
+        <v>8</v>
       </c>
       <c r="I3" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="J3" s="11" t="inlineStr">
-        <is>
           <t>On track</t>
         </is>
       </c>
-      <c r="K3" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L3" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M3" s="12" t="inlineStr">
-        <is>
-          <t>Pairing on auth Thursday. Keep the momentum.</t>
+      <c r="J3" s="12" t="inlineStr">
+        <is>
+          <t>Strong week. Pair on auth Thursday.</t>
         </is>
       </c>
     </row>
@@ -993,41 +979,30 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E4" s="11" t="n">
-        <v>41</v>
-      </c>
-      <c r="F4" s="11" t="n">
-        <v>79</v>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>Component composition, responsive dashboard</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>Dashboard in (late), composition reading done</t>
+        </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>58</v>
-      </c>
-      <c r="H4" s="11" t="inlineStr">
-        <is>
-          <t>Up</t>
-        </is>
+        <v>60</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>6</v>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="J4" s="11" t="inlineStr">
-        <is>
           <t>Watch</t>
         </is>
       </c>
-      <c r="K4" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="L4" s="11" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M4" s="12" t="inlineStr">
-        <is>
-          <t>Protect deadlines, shift due times to AM PKT.</t>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>Good effort against real constraints. Protect deadlines.</t>
         </is>
       </c>
     </row>
@@ -1050,41 +1025,30 @@
           <t>Excused</t>
         </is>
       </c>
-      <c r="E5" s="11" t="n">
-        <v>31</v>
-      </c>
-      <c r="F5" s="11" t="n">
-        <v>34</v>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>API integration, REST best-practices reading</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>Little progress, re-engaging</t>
+        </is>
       </c>
       <c r="G5" s="11" t="n">
-        <v>44</v>
-      </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>Down</t>
-        </is>
+        <v>20</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>3</v>
       </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J5" s="11" t="inlineStr">
-        <is>
           <t>At risk</t>
         </is>
       </c>
-      <c r="K5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M5" s="12" t="inlineStr">
-        <is>
-          <t>Warm check-in done. Re-engage gently, small wins first.</t>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>Warm check-in done. Small wins first, light load next week.</t>
         </is>
       </c>
     </row>
@@ -1107,41 +1071,30 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E6" s="11" t="n">
-        <v>95</v>
-      </c>
-      <c r="F6" s="11" t="n">
-        <v>76</v>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>Auth middleware, rate-limiting stretch</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>Auth middleware done early</t>
+        </is>
       </c>
       <c r="G6" s="11" t="n">
-        <v>97</v>
-      </c>
-      <c r="H6" s="11" t="inlineStr">
-        <is>
-          <t>Flat</t>
-        </is>
+        <v>100</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>9</v>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="J6" s="11" t="inlineStr">
-        <is>
           <t>On track</t>
         </is>
       </c>
-      <c r="K6" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="11" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M6" s="12" t="inlineStr">
-        <is>
-          <t>Add a stretch track so he is challenged.</t>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>Way ahead. Add a real stretch so he is challenged.</t>
         </is>
       </c>
     </row>
@@ -1164,41 +1117,30 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E7" s="11" t="n">
-        <v>64</v>
-      </c>
-      <c r="F7" s="11" t="n">
-        <v>71</v>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>Async/await refactor, event loop reading</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>Refactor in progress, reading done</t>
+        </is>
       </c>
       <c r="G7" s="11" t="n">
-        <v>79</v>
-      </c>
-      <c r="H7" s="11" t="inlineStr">
-        <is>
-          <t>Up</t>
-        </is>
+        <v>75</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>8</v>
       </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="J7" s="11" t="inlineStr">
-        <is>
           <t>On track</t>
         </is>
       </c>
-      <c r="K7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L7" s="11" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M7" s="12" t="inlineStr">
-        <is>
-          <t>Unblock async/await, then keep the climb going.</t>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>Climbing nicely. Unblock async/await and keep going.</t>
         </is>
       </c>
     </row>
@@ -1221,41 +1163,30 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E8" s="11" t="n">
-        <v>53</v>
-      </c>
-      <c r="F8" s="11" t="n">
-        <v>49</v>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>Validation library, regex quiz</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>Library in (late), quiz pending</t>
+        </is>
       </c>
       <c r="G8" s="11" t="n">
-        <v>62</v>
-      </c>
-      <c r="H8" s="11" t="inlineStr">
-        <is>
-          <t>Down</t>
-        </is>
+        <v>55</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>5</v>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="J8" s="11" t="inlineStr">
-        <is>
           <t>Watch</t>
         </is>
       </c>
-      <c r="K8" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L8" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M8" s="12" t="inlineStr">
-        <is>
-          <t>Short check-in this week before it slides further.</t>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>Slipping a little. Short check-in this week.</t>
         </is>
       </c>
     </row>
@@ -1281,15 +1212,12 @@
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr"/>
-      <c r="E10" s="11" t="inlineStr"/>
-      <c r="F10" s="11" t="inlineStr"/>
+      <c r="E10" s="12" t="inlineStr"/>
+      <c r="F10" s="12" t="inlineStr"/>
       <c r="G10" s="11" t="inlineStr"/>
       <c r="H10" s="11" t="inlineStr"/>
       <c r="I10" s="11" t="inlineStr"/>
-      <c r="J10" s="11" t="inlineStr"/>
-      <c r="K10" s="11" t="inlineStr"/>
-      <c r="L10" s="11" t="inlineStr"/>
-      <c r="M10" s="12" t="inlineStr"/>
+      <c r="J10" s="12" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n">
@@ -1306,15 +1234,12 @@
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr"/>
-      <c r="E11" s="11" t="inlineStr"/>
-      <c r="F11" s="11" t="inlineStr"/>
+      <c r="E11" s="12" t="inlineStr"/>
+      <c r="F11" s="12" t="inlineStr"/>
       <c r="G11" s="11" t="inlineStr"/>
       <c r="H11" s="11" t="inlineStr"/>
       <c r="I11" s="11" t="inlineStr"/>
-      <c r="J11" s="11" t="inlineStr"/>
-      <c r="K11" s="11" t="inlineStr"/>
-      <c r="L11" s="11" t="inlineStr"/>
-      <c r="M11" s="12" t="inlineStr"/>
+      <c r="J11" s="12" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n">
@@ -1331,15 +1256,12 @@
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr"/>
-      <c r="E12" s="11" t="inlineStr"/>
-      <c r="F12" s="11" t="inlineStr"/>
+      <c r="E12" s="12" t="inlineStr"/>
+      <c r="F12" s="12" t="inlineStr"/>
       <c r="G12" s="11" t="inlineStr"/>
       <c r="H12" s="11" t="inlineStr"/>
       <c r="I12" s="11" t="inlineStr"/>
-      <c r="J12" s="11" t="inlineStr"/>
-      <c r="K12" s="11" t="inlineStr"/>
-      <c r="L12" s="11" t="inlineStr"/>
-      <c r="M12" s="12" t="inlineStr"/>
+      <c r="J12" s="12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n">
@@ -1356,15 +1278,12 @@
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr"/>
-      <c r="E13" s="11" t="inlineStr"/>
-      <c r="F13" s="11" t="inlineStr"/>
+      <c r="E13" s="12" t="inlineStr"/>
+      <c r="F13" s="12" t="inlineStr"/>
       <c r="G13" s="11" t="inlineStr"/>
       <c r="H13" s="11" t="inlineStr"/>
       <c r="I13" s="11" t="inlineStr"/>
-      <c r="J13" s="11" t="inlineStr"/>
-      <c r="K13" s="11" t="inlineStr"/>
-      <c r="L13" s="11" t="inlineStr"/>
-      <c r="M13" s="12" t="inlineStr"/>
+      <c r="J13" s="12" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="n">
@@ -1381,15 +1300,12 @@
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr"/>
-      <c r="E14" s="11" t="inlineStr"/>
-      <c r="F14" s="11" t="inlineStr"/>
+      <c r="E14" s="12" t="inlineStr"/>
+      <c r="F14" s="12" t="inlineStr"/>
       <c r="G14" s="11" t="inlineStr"/>
       <c r="H14" s="11" t="inlineStr"/>
       <c r="I14" s="11" t="inlineStr"/>
-      <c r="J14" s="11" t="inlineStr"/>
-      <c r="K14" s="11" t="inlineStr"/>
-      <c r="L14" s="11" t="inlineStr"/>
-      <c r="M14" s="12" t="inlineStr"/>
+      <c r="J14" s="12" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n">
@@ -1406,15 +1322,12 @@
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr"/>
-      <c r="E15" s="11" t="inlineStr"/>
-      <c r="F15" s="11" t="inlineStr"/>
+      <c r="E15" s="12" t="inlineStr"/>
+      <c r="F15" s="12" t="inlineStr"/>
       <c r="G15" s="11" t="inlineStr"/>
       <c r="H15" s="11" t="inlineStr"/>
       <c r="I15" s="11" t="inlineStr"/>
-      <c r="J15" s="11" t="inlineStr"/>
-      <c r="K15" s="11" t="inlineStr"/>
-      <c r="L15" s="11" t="inlineStr"/>
-      <c r="M15" s="12" t="inlineStr"/>
+      <c r="J15" s="12" t="inlineStr"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -1438,15 +1351,12 @@
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr"/>
-      <c r="E17" s="11" t="inlineStr"/>
-      <c r="F17" s="11" t="inlineStr"/>
+      <c r="E17" s="12" t="inlineStr"/>
+      <c r="F17" s="12" t="inlineStr"/>
       <c r="G17" s="11" t="inlineStr"/>
       <c r="H17" s="11" t="inlineStr"/>
       <c r="I17" s="11" t="inlineStr"/>
-      <c r="J17" s="11" t="inlineStr"/>
-      <c r="K17" s="11" t="inlineStr"/>
-      <c r="L17" s="11" t="inlineStr"/>
-      <c r="M17" s="12" t="inlineStr"/>
+      <c r="J17" s="12" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="n">
@@ -1463,15 +1373,12 @@
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr"/>
-      <c r="E18" s="11" t="inlineStr"/>
-      <c r="F18" s="11" t="inlineStr"/>
+      <c r="E18" s="12" t="inlineStr"/>
+      <c r="F18" s="12" t="inlineStr"/>
       <c r="G18" s="11" t="inlineStr"/>
       <c r="H18" s="11" t="inlineStr"/>
       <c r="I18" s="11" t="inlineStr"/>
-      <c r="J18" s="11" t="inlineStr"/>
-      <c r="K18" s="11" t="inlineStr"/>
-      <c r="L18" s="11" t="inlineStr"/>
-      <c r="M18" s="12" t="inlineStr"/>
+      <c r="J18" s="12" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="n">
@@ -1488,15 +1395,12 @@
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr"/>
-      <c r="E19" s="11" t="inlineStr"/>
-      <c r="F19" s="11" t="inlineStr"/>
+      <c r="E19" s="12" t="inlineStr"/>
+      <c r="F19" s="12" t="inlineStr"/>
       <c r="G19" s="11" t="inlineStr"/>
       <c r="H19" s="11" t="inlineStr"/>
       <c r="I19" s="11" t="inlineStr"/>
-      <c r="J19" s="11" t="inlineStr"/>
-      <c r="K19" s="11" t="inlineStr"/>
-      <c r="L19" s="11" t="inlineStr"/>
-      <c r="M19" s="12" t="inlineStr"/>
+      <c r="J19" s="12" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="n">
@@ -1513,15 +1417,12 @@
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr"/>
-      <c r="E20" s="11" t="inlineStr"/>
-      <c r="F20" s="11" t="inlineStr"/>
+      <c r="E20" s="12" t="inlineStr"/>
+      <c r="F20" s="12" t="inlineStr"/>
       <c r="G20" s="11" t="inlineStr"/>
       <c r="H20" s="11" t="inlineStr"/>
       <c r="I20" s="11" t="inlineStr"/>
-      <c r="J20" s="11" t="inlineStr"/>
-      <c r="K20" s="11" t="inlineStr"/>
-      <c r="L20" s="11" t="inlineStr"/>
-      <c r="M20" s="12" t="inlineStr"/>
+      <c r="J20" s="12" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="9" t="n">
@@ -1538,15 +1439,12 @@
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr"/>
-      <c r="E21" s="11" t="inlineStr"/>
-      <c r="F21" s="11" t="inlineStr"/>
+      <c r="E21" s="12" t="inlineStr"/>
+      <c r="F21" s="12" t="inlineStr"/>
       <c r="G21" s="11" t="inlineStr"/>
       <c r="H21" s="11" t="inlineStr"/>
       <c r="I21" s="11" t="inlineStr"/>
-      <c r="J21" s="11" t="inlineStr"/>
-      <c r="K21" s="11" t="inlineStr"/>
-      <c r="L21" s="11" t="inlineStr"/>
-      <c r="M21" s="12" t="inlineStr"/>
+      <c r="J21" s="12" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="9" t="n">
@@ -1563,15 +1461,12 @@
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr"/>
-      <c r="E22" s="11" t="inlineStr"/>
-      <c r="F22" s="11" t="inlineStr"/>
+      <c r="E22" s="12" t="inlineStr"/>
+      <c r="F22" s="12" t="inlineStr"/>
       <c r="G22" s="11" t="inlineStr"/>
       <c r="H22" s="11" t="inlineStr"/>
       <c r="I22" s="11" t="inlineStr"/>
-      <c r="J22" s="11" t="inlineStr"/>
-      <c r="K22" s="11" t="inlineStr"/>
-      <c r="L22" s="11" t="inlineStr"/>
-      <c r="M22" s="12" t="inlineStr"/>
+      <c r="J22" s="12" t="inlineStr"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
@@ -1595,15 +1490,12 @@
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr"/>
-      <c r="E24" s="11" t="inlineStr"/>
-      <c r="F24" s="11" t="inlineStr"/>
+      <c r="E24" s="12" t="inlineStr"/>
+      <c r="F24" s="12" t="inlineStr"/>
       <c r="G24" s="11" t="inlineStr"/>
       <c r="H24" s="11" t="inlineStr"/>
       <c r="I24" s="11" t="inlineStr"/>
-      <c r="J24" s="11" t="inlineStr"/>
-      <c r="K24" s="11" t="inlineStr"/>
-      <c r="L24" s="11" t="inlineStr"/>
-      <c r="M24" s="12" t="inlineStr"/>
+      <c r="J24" s="12" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="9" t="n">
@@ -1620,15 +1512,12 @@
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr"/>
-      <c r="E25" s="11" t="inlineStr"/>
-      <c r="F25" s="11" t="inlineStr"/>
+      <c r="E25" s="12" t="inlineStr"/>
+      <c r="F25" s="12" t="inlineStr"/>
       <c r="G25" s="11" t="inlineStr"/>
       <c r="H25" s="11" t="inlineStr"/>
       <c r="I25" s="11" t="inlineStr"/>
-      <c r="J25" s="11" t="inlineStr"/>
-      <c r="K25" s="11" t="inlineStr"/>
-      <c r="L25" s="11" t="inlineStr"/>
-      <c r="M25" s="12" t="inlineStr"/>
+      <c r="J25" s="12" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="9" t="n">
@@ -1645,15 +1534,12 @@
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr"/>
-      <c r="E26" s="11" t="inlineStr"/>
-      <c r="F26" s="11" t="inlineStr"/>
+      <c r="E26" s="12" t="inlineStr"/>
+      <c r="F26" s="12" t="inlineStr"/>
       <c r="G26" s="11" t="inlineStr"/>
       <c r="H26" s="11" t="inlineStr"/>
       <c r="I26" s="11" t="inlineStr"/>
-      <c r="J26" s="11" t="inlineStr"/>
-      <c r="K26" s="11" t="inlineStr"/>
-      <c r="L26" s="11" t="inlineStr"/>
-      <c r="M26" s="12" t="inlineStr"/>
+      <c r="J26" s="12" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="9" t="n">
@@ -1670,15 +1556,12 @@
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr"/>
-      <c r="E27" s="11" t="inlineStr"/>
-      <c r="F27" s="11" t="inlineStr"/>
+      <c r="E27" s="12" t="inlineStr"/>
+      <c r="F27" s="12" t="inlineStr"/>
       <c r="G27" s="11" t="inlineStr"/>
       <c r="H27" s="11" t="inlineStr"/>
       <c r="I27" s="11" t="inlineStr"/>
-      <c r="J27" s="11" t="inlineStr"/>
-      <c r="K27" s="11" t="inlineStr"/>
-      <c r="L27" s="11" t="inlineStr"/>
-      <c r="M27" s="12" t="inlineStr"/>
+      <c r="J27" s="12" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="9" t="n">
@@ -1695,15 +1578,12 @@
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr"/>
-      <c r="E28" s="11" t="inlineStr"/>
-      <c r="F28" s="11" t="inlineStr"/>
+      <c r="E28" s="12" t="inlineStr"/>
+      <c r="F28" s="12" t="inlineStr"/>
       <c r="G28" s="11" t="inlineStr"/>
       <c r="H28" s="11" t="inlineStr"/>
       <c r="I28" s="11" t="inlineStr"/>
-      <c r="J28" s="11" t="inlineStr"/>
-      <c r="K28" s="11" t="inlineStr"/>
-      <c r="L28" s="11" t="inlineStr"/>
-      <c r="M28" s="12" t="inlineStr"/>
+      <c r="J28" s="12" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n">
@@ -1720,15 +1600,12 @@
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr"/>
-      <c r="E29" s="11" t="inlineStr"/>
-      <c r="F29" s="11" t="inlineStr"/>
+      <c r="E29" s="12" t="inlineStr"/>
+      <c r="F29" s="12" t="inlineStr"/>
       <c r="G29" s="11" t="inlineStr"/>
       <c r="H29" s="11" t="inlineStr"/>
       <c r="I29" s="11" t="inlineStr"/>
-      <c r="J29" s="11" t="inlineStr"/>
-      <c r="K29" s="11" t="inlineStr"/>
-      <c r="L29" s="11" t="inlineStr"/>
-      <c r="M29" s="12" t="inlineStr"/>
+      <c r="J29" s="12" t="inlineStr"/>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
@@ -1752,15 +1629,12 @@
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr"/>
-      <c r="E31" s="11" t="inlineStr"/>
-      <c r="F31" s="11" t="inlineStr"/>
+      <c r="E31" s="12" t="inlineStr"/>
+      <c r="F31" s="12" t="inlineStr"/>
       <c r="G31" s="11" t="inlineStr"/>
       <c r="H31" s="11" t="inlineStr"/>
       <c r="I31" s="11" t="inlineStr"/>
-      <c r="J31" s="11" t="inlineStr"/>
-      <c r="K31" s="11" t="inlineStr"/>
-      <c r="L31" s="11" t="inlineStr"/>
-      <c r="M31" s="12" t="inlineStr"/>
+      <c r="J31" s="12" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="9" t="n">
@@ -1777,15 +1651,12 @@
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr"/>
-      <c r="E32" s="11" t="inlineStr"/>
-      <c r="F32" s="11" t="inlineStr"/>
+      <c r="E32" s="12" t="inlineStr"/>
+      <c r="F32" s="12" t="inlineStr"/>
       <c r="G32" s="11" t="inlineStr"/>
       <c r="H32" s="11" t="inlineStr"/>
       <c r="I32" s="11" t="inlineStr"/>
-      <c r="J32" s="11" t="inlineStr"/>
-      <c r="K32" s="11" t="inlineStr"/>
-      <c r="L32" s="11" t="inlineStr"/>
-      <c r="M32" s="12" t="inlineStr"/>
+      <c r="J32" s="12" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="9" t="n">
@@ -1802,15 +1673,12 @@
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr"/>
-      <c r="E33" s="11" t="inlineStr"/>
-      <c r="F33" s="11" t="inlineStr"/>
+      <c r="E33" s="12" t="inlineStr"/>
+      <c r="F33" s="12" t="inlineStr"/>
       <c r="G33" s="11" t="inlineStr"/>
       <c r="H33" s="11" t="inlineStr"/>
       <c r="I33" s="11" t="inlineStr"/>
-      <c r="J33" s="11" t="inlineStr"/>
-      <c r="K33" s="11" t="inlineStr"/>
-      <c r="L33" s="11" t="inlineStr"/>
-      <c r="M33" s="12" t="inlineStr"/>
+      <c r="J33" s="12" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="9" t="n">
@@ -1827,15 +1695,12 @@
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr"/>
-      <c r="E34" s="11" t="inlineStr"/>
-      <c r="F34" s="11" t="inlineStr"/>
+      <c r="E34" s="12" t="inlineStr"/>
+      <c r="F34" s="12" t="inlineStr"/>
       <c r="G34" s="11" t="inlineStr"/>
       <c r="H34" s="11" t="inlineStr"/>
       <c r="I34" s="11" t="inlineStr"/>
-      <c r="J34" s="11" t="inlineStr"/>
-      <c r="K34" s="11" t="inlineStr"/>
-      <c r="L34" s="11" t="inlineStr"/>
-      <c r="M34" s="12" t="inlineStr"/>
+      <c r="J34" s="12" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="9" t="n">
@@ -1852,15 +1717,12 @@
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr"/>
-      <c r="E35" s="11" t="inlineStr"/>
-      <c r="F35" s="11" t="inlineStr"/>
+      <c r="E35" s="12" t="inlineStr"/>
+      <c r="F35" s="12" t="inlineStr"/>
       <c r="G35" s="11" t="inlineStr"/>
       <c r="H35" s="11" t="inlineStr"/>
       <c r="I35" s="11" t="inlineStr"/>
-      <c r="J35" s="11" t="inlineStr"/>
-      <c r="K35" s="11" t="inlineStr"/>
-      <c r="L35" s="11" t="inlineStr"/>
-      <c r="M35" s="12" t="inlineStr"/>
+      <c r="J35" s="12" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="9" t="n">
@@ -1877,15 +1739,12 @@
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr"/>
-      <c r="E36" s="11" t="inlineStr"/>
-      <c r="F36" s="11" t="inlineStr"/>
+      <c r="E36" s="12" t="inlineStr"/>
+      <c r="F36" s="12" t="inlineStr"/>
       <c r="G36" s="11" t="inlineStr"/>
       <c r="H36" s="11" t="inlineStr"/>
       <c r="I36" s="11" t="inlineStr"/>
-      <c r="J36" s="11" t="inlineStr"/>
-      <c r="K36" s="11" t="inlineStr"/>
-      <c r="L36" s="11" t="inlineStr"/>
-      <c r="M36" s="12" t="inlineStr"/>
+      <c r="J36" s="12" t="inlineStr"/>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="8" t="inlineStr">
@@ -1909,15 +1768,12 @@
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr"/>
-      <c r="E38" s="11" t="inlineStr"/>
-      <c r="F38" s="11" t="inlineStr"/>
+      <c r="E38" s="12" t="inlineStr"/>
+      <c r="F38" s="12" t="inlineStr"/>
       <c r="G38" s="11" t="inlineStr"/>
       <c r="H38" s="11" t="inlineStr"/>
       <c r="I38" s="11" t="inlineStr"/>
-      <c r="J38" s="11" t="inlineStr"/>
-      <c r="K38" s="11" t="inlineStr"/>
-      <c r="L38" s="11" t="inlineStr"/>
-      <c r="M38" s="12" t="inlineStr"/>
+      <c r="J38" s="12" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="9" t="n">
@@ -1934,15 +1790,12 @@
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr"/>
-      <c r="E39" s="11" t="inlineStr"/>
-      <c r="F39" s="11" t="inlineStr"/>
+      <c r="E39" s="12" t="inlineStr"/>
+      <c r="F39" s="12" t="inlineStr"/>
       <c r="G39" s="11" t="inlineStr"/>
       <c r="H39" s="11" t="inlineStr"/>
       <c r="I39" s="11" t="inlineStr"/>
-      <c r="J39" s="11" t="inlineStr"/>
-      <c r="K39" s="11" t="inlineStr"/>
-      <c r="L39" s="11" t="inlineStr"/>
-      <c r="M39" s="12" t="inlineStr"/>
+      <c r="J39" s="12" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="9" t="n">
@@ -1959,15 +1812,12 @@
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr"/>
-      <c r="E40" s="11" t="inlineStr"/>
-      <c r="F40" s="11" t="inlineStr"/>
+      <c r="E40" s="12" t="inlineStr"/>
+      <c r="F40" s="12" t="inlineStr"/>
       <c r="G40" s="11" t="inlineStr"/>
       <c r="H40" s="11" t="inlineStr"/>
       <c r="I40" s="11" t="inlineStr"/>
-      <c r="J40" s="11" t="inlineStr"/>
-      <c r="K40" s="11" t="inlineStr"/>
-      <c r="L40" s="11" t="inlineStr"/>
-      <c r="M40" s="12" t="inlineStr"/>
+      <c r="J40" s="12" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="9" t="n">
@@ -1984,15 +1834,12 @@
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr"/>
-      <c r="E41" s="11" t="inlineStr"/>
-      <c r="F41" s="11" t="inlineStr"/>
+      <c r="E41" s="12" t="inlineStr"/>
+      <c r="F41" s="12" t="inlineStr"/>
       <c r="G41" s="11" t="inlineStr"/>
       <c r="H41" s="11" t="inlineStr"/>
       <c r="I41" s="11" t="inlineStr"/>
-      <c r="J41" s="11" t="inlineStr"/>
-      <c r="K41" s="11" t="inlineStr"/>
-      <c r="L41" s="11" t="inlineStr"/>
-      <c r="M41" s="12" t="inlineStr"/>
+      <c r="J41" s="12" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="9" t="n">
@@ -2009,15 +1856,12 @@
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr"/>
-      <c r="E42" s="11" t="inlineStr"/>
-      <c r="F42" s="11" t="inlineStr"/>
+      <c r="E42" s="12" t="inlineStr"/>
+      <c r="F42" s="12" t="inlineStr"/>
       <c r="G42" s="11" t="inlineStr"/>
       <c r="H42" s="11" t="inlineStr"/>
       <c r="I42" s="11" t="inlineStr"/>
-      <c r="J42" s="11" t="inlineStr"/>
-      <c r="K42" s="11" t="inlineStr"/>
-      <c r="L42" s="11" t="inlineStr"/>
-      <c r="M42" s="12" t="inlineStr"/>
+      <c r="J42" s="12" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="9" t="n">
@@ -2034,15 +1878,12 @@
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr"/>
-      <c r="E43" s="11" t="inlineStr"/>
-      <c r="F43" s="11" t="inlineStr"/>
+      <c r="E43" s="12" t="inlineStr"/>
+      <c r="F43" s="12" t="inlineStr"/>
       <c r="G43" s="11" t="inlineStr"/>
       <c r="H43" s="11" t="inlineStr"/>
       <c r="I43" s="11" t="inlineStr"/>
-      <c r="J43" s="11" t="inlineStr"/>
-      <c r="K43" s="11" t="inlineStr"/>
-      <c r="L43" s="11" t="inlineStr"/>
-      <c r="M43" s="12" t="inlineStr"/>
+      <c r="J43" s="12" t="inlineStr"/>
     </row>
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="8" t="inlineStr">
@@ -2066,15 +1907,12 @@
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr"/>
-      <c r="E45" s="11" t="inlineStr"/>
-      <c r="F45" s="11" t="inlineStr"/>
+      <c r="E45" s="12" t="inlineStr"/>
+      <c r="F45" s="12" t="inlineStr"/>
       <c r="G45" s="11" t="inlineStr"/>
       <c r="H45" s="11" t="inlineStr"/>
       <c r="I45" s="11" t="inlineStr"/>
-      <c r="J45" s="11" t="inlineStr"/>
-      <c r="K45" s="11" t="inlineStr"/>
-      <c r="L45" s="11" t="inlineStr"/>
-      <c r="M45" s="12" t="inlineStr"/>
+      <c r="J45" s="12" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="9" t="n">
@@ -2091,15 +1929,12 @@
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr"/>
-      <c r="E46" s="11" t="inlineStr"/>
-      <c r="F46" s="11" t="inlineStr"/>
+      <c r="E46" s="12" t="inlineStr"/>
+      <c r="F46" s="12" t="inlineStr"/>
       <c r="G46" s="11" t="inlineStr"/>
       <c r="H46" s="11" t="inlineStr"/>
       <c r="I46" s="11" t="inlineStr"/>
-      <c r="J46" s="11" t="inlineStr"/>
-      <c r="K46" s="11" t="inlineStr"/>
-      <c r="L46" s="11" t="inlineStr"/>
-      <c r="M46" s="12" t="inlineStr"/>
+      <c r="J46" s="12" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="9" t="n">
@@ -2116,15 +1951,12 @@
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr"/>
-      <c r="E47" s="11" t="inlineStr"/>
-      <c r="F47" s="11" t="inlineStr"/>
+      <c r="E47" s="12" t="inlineStr"/>
+      <c r="F47" s="12" t="inlineStr"/>
       <c r="G47" s="11" t="inlineStr"/>
       <c r="H47" s="11" t="inlineStr"/>
       <c r="I47" s="11" t="inlineStr"/>
-      <c r="J47" s="11" t="inlineStr"/>
-      <c r="K47" s="11" t="inlineStr"/>
-      <c r="L47" s="11" t="inlineStr"/>
-      <c r="M47" s="12" t="inlineStr"/>
+      <c r="J47" s="12" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="9" t="n">
@@ -2141,15 +1973,12 @@
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr"/>
-      <c r="E48" s="11" t="inlineStr"/>
-      <c r="F48" s="11" t="inlineStr"/>
+      <c r="E48" s="12" t="inlineStr"/>
+      <c r="F48" s="12" t="inlineStr"/>
       <c r="G48" s="11" t="inlineStr"/>
       <c r="H48" s="11" t="inlineStr"/>
       <c r="I48" s="11" t="inlineStr"/>
-      <c r="J48" s="11" t="inlineStr"/>
-      <c r="K48" s="11" t="inlineStr"/>
-      <c r="L48" s="11" t="inlineStr"/>
-      <c r="M48" s="12" t="inlineStr"/>
+      <c r="J48" s="12" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="9" t="n">
@@ -2166,15 +1995,12 @@
         </is>
       </c>
       <c r="D49" s="11" t="inlineStr"/>
-      <c r="E49" s="11" t="inlineStr"/>
-      <c r="F49" s="11" t="inlineStr"/>
+      <c r="E49" s="12" t="inlineStr"/>
+      <c r="F49" s="12" t="inlineStr"/>
       <c r="G49" s="11" t="inlineStr"/>
       <c r="H49" s="11" t="inlineStr"/>
       <c r="I49" s="11" t="inlineStr"/>
-      <c r="J49" s="11" t="inlineStr"/>
-      <c r="K49" s="11" t="inlineStr"/>
-      <c r="L49" s="11" t="inlineStr"/>
-      <c r="M49" s="12" t="inlineStr"/>
+      <c r="J49" s="12" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="9" t="n">
@@ -2191,15 +2017,12 @@
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr"/>
-      <c r="E50" s="11" t="inlineStr"/>
-      <c r="F50" s="11" t="inlineStr"/>
+      <c r="E50" s="12" t="inlineStr"/>
+      <c r="F50" s="12" t="inlineStr"/>
       <c r="G50" s="11" t="inlineStr"/>
       <c r="H50" s="11" t="inlineStr"/>
       <c r="I50" s="11" t="inlineStr"/>
-      <c r="J50" s="11" t="inlineStr"/>
-      <c r="K50" s="11" t="inlineStr"/>
-      <c r="L50" s="11" t="inlineStr"/>
-      <c r="M50" s="12" t="inlineStr"/>
+      <c r="J50" s="12" t="inlineStr"/>
     </row>
     <row r="51" ht="22" customHeight="1">
       <c r="A51" s="8" t="inlineStr">
@@ -2223,15 +2046,12 @@
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr"/>
-      <c r="E52" s="11" t="inlineStr"/>
-      <c r="F52" s="11" t="inlineStr"/>
+      <c r="E52" s="12" t="inlineStr"/>
+      <c r="F52" s="12" t="inlineStr"/>
       <c r="G52" s="11" t="inlineStr"/>
       <c r="H52" s="11" t="inlineStr"/>
       <c r="I52" s="11" t="inlineStr"/>
-      <c r="J52" s="11" t="inlineStr"/>
-      <c r="K52" s="11" t="inlineStr"/>
-      <c r="L52" s="11" t="inlineStr"/>
-      <c r="M52" s="12" t="inlineStr"/>
+      <c r="J52" s="12" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="9" t="n">
@@ -2248,15 +2068,12 @@
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr"/>
-      <c r="E53" s="11" t="inlineStr"/>
-      <c r="F53" s="11" t="inlineStr"/>
+      <c r="E53" s="12" t="inlineStr"/>
+      <c r="F53" s="12" t="inlineStr"/>
       <c r="G53" s="11" t="inlineStr"/>
       <c r="H53" s="11" t="inlineStr"/>
       <c r="I53" s="11" t="inlineStr"/>
-      <c r="J53" s="11" t="inlineStr"/>
-      <c r="K53" s="11" t="inlineStr"/>
-      <c r="L53" s="11" t="inlineStr"/>
-      <c r="M53" s="12" t="inlineStr"/>
+      <c r="J53" s="12" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="9" t="n">
@@ -2273,15 +2090,12 @@
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr"/>
-      <c r="E54" s="11" t="inlineStr"/>
-      <c r="F54" s="11" t="inlineStr"/>
+      <c r="E54" s="12" t="inlineStr"/>
+      <c r="F54" s="12" t="inlineStr"/>
       <c r="G54" s="11" t="inlineStr"/>
       <c r="H54" s="11" t="inlineStr"/>
       <c r="I54" s="11" t="inlineStr"/>
-      <c r="J54" s="11" t="inlineStr"/>
-      <c r="K54" s="11" t="inlineStr"/>
-      <c r="L54" s="11" t="inlineStr"/>
-      <c r="M54" s="12" t="inlineStr"/>
+      <c r="J54" s="12" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="9" t="n">
@@ -2298,15 +2112,12 @@
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr"/>
-      <c r="E55" s="11" t="inlineStr"/>
-      <c r="F55" s="11" t="inlineStr"/>
+      <c r="E55" s="12" t="inlineStr"/>
+      <c r="F55" s="12" t="inlineStr"/>
       <c r="G55" s="11" t="inlineStr"/>
       <c r="H55" s="11" t="inlineStr"/>
       <c r="I55" s="11" t="inlineStr"/>
-      <c r="J55" s="11" t="inlineStr"/>
-      <c r="K55" s="11" t="inlineStr"/>
-      <c r="L55" s="11" t="inlineStr"/>
-      <c r="M55" s="12" t="inlineStr"/>
+      <c r="J55" s="12" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="9" t="n">
@@ -2323,15 +2134,12 @@
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr"/>
-      <c r="E56" s="11" t="inlineStr"/>
-      <c r="F56" s="11" t="inlineStr"/>
+      <c r="E56" s="12" t="inlineStr"/>
+      <c r="F56" s="12" t="inlineStr"/>
       <c r="G56" s="11" t="inlineStr"/>
       <c r="H56" s="11" t="inlineStr"/>
       <c r="I56" s="11" t="inlineStr"/>
-      <c r="J56" s="11" t="inlineStr"/>
-      <c r="K56" s="11" t="inlineStr"/>
-      <c r="L56" s="11" t="inlineStr"/>
-      <c r="M56" s="12" t="inlineStr"/>
+      <c r="J56" s="12" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="9" t="n">
@@ -2348,15 +2156,12 @@
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr"/>
-      <c r="E57" s="11" t="inlineStr"/>
-      <c r="F57" s="11" t="inlineStr"/>
+      <c r="E57" s="12" t="inlineStr"/>
+      <c r="F57" s="12" t="inlineStr"/>
       <c r="G57" s="11" t="inlineStr"/>
       <c r="H57" s="11" t="inlineStr"/>
       <c r="I57" s="11" t="inlineStr"/>
-      <c r="J57" s="11" t="inlineStr"/>
-      <c r="K57" s="11" t="inlineStr"/>
-      <c r="L57" s="11" t="inlineStr"/>
-      <c r="M57" s="12" t="inlineStr"/>
+      <c r="J57" s="12" t="inlineStr"/>
     </row>
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="8" t="inlineStr">
@@ -2380,15 +2185,12 @@
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr"/>
-      <c r="E59" s="11" t="inlineStr"/>
-      <c r="F59" s="11" t="inlineStr"/>
+      <c r="E59" s="12" t="inlineStr"/>
+      <c r="F59" s="12" t="inlineStr"/>
       <c r="G59" s="11" t="inlineStr"/>
       <c r="H59" s="11" t="inlineStr"/>
       <c r="I59" s="11" t="inlineStr"/>
-      <c r="J59" s="11" t="inlineStr"/>
-      <c r="K59" s="11" t="inlineStr"/>
-      <c r="L59" s="11" t="inlineStr"/>
-      <c r="M59" s="12" t="inlineStr"/>
+      <c r="J59" s="12" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="9" t="n">
@@ -2405,15 +2207,12 @@
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr"/>
-      <c r="E60" s="11" t="inlineStr"/>
-      <c r="F60" s="11" t="inlineStr"/>
+      <c r="E60" s="12" t="inlineStr"/>
+      <c r="F60" s="12" t="inlineStr"/>
       <c r="G60" s="11" t="inlineStr"/>
       <c r="H60" s="11" t="inlineStr"/>
       <c r="I60" s="11" t="inlineStr"/>
-      <c r="J60" s="11" t="inlineStr"/>
-      <c r="K60" s="11" t="inlineStr"/>
-      <c r="L60" s="11" t="inlineStr"/>
-      <c r="M60" s="12" t="inlineStr"/>
+      <c r="J60" s="12" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="9" t="n">
@@ -2430,15 +2229,12 @@
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr"/>
-      <c r="E61" s="11" t="inlineStr"/>
-      <c r="F61" s="11" t="inlineStr"/>
+      <c r="E61" s="12" t="inlineStr"/>
+      <c r="F61" s="12" t="inlineStr"/>
       <c r="G61" s="11" t="inlineStr"/>
       <c r="H61" s="11" t="inlineStr"/>
       <c r="I61" s="11" t="inlineStr"/>
-      <c r="J61" s="11" t="inlineStr"/>
-      <c r="K61" s="11" t="inlineStr"/>
-      <c r="L61" s="11" t="inlineStr"/>
-      <c r="M61" s="12" t="inlineStr"/>
+      <c r="J61" s="12" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="9" t="n">
@@ -2455,15 +2251,12 @@
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr"/>
-      <c r="E62" s="11" t="inlineStr"/>
-      <c r="F62" s="11" t="inlineStr"/>
+      <c r="E62" s="12" t="inlineStr"/>
+      <c r="F62" s="12" t="inlineStr"/>
       <c r="G62" s="11" t="inlineStr"/>
       <c r="H62" s="11" t="inlineStr"/>
       <c r="I62" s="11" t="inlineStr"/>
-      <c r="J62" s="11" t="inlineStr"/>
-      <c r="K62" s="11" t="inlineStr"/>
-      <c r="L62" s="11" t="inlineStr"/>
-      <c r="M62" s="12" t="inlineStr"/>
+      <c r="J62" s="12" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="9" t="n">
@@ -2480,15 +2273,12 @@
         </is>
       </c>
       <c r="D63" s="11" t="inlineStr"/>
-      <c r="E63" s="11" t="inlineStr"/>
-      <c r="F63" s="11" t="inlineStr"/>
+      <c r="E63" s="12" t="inlineStr"/>
+      <c r="F63" s="12" t="inlineStr"/>
       <c r="G63" s="11" t="inlineStr"/>
       <c r="H63" s="11" t="inlineStr"/>
       <c r="I63" s="11" t="inlineStr"/>
-      <c r="J63" s="11" t="inlineStr"/>
-      <c r="K63" s="11" t="inlineStr"/>
-      <c r="L63" s="11" t="inlineStr"/>
-      <c r="M63" s="12" t="inlineStr"/>
+      <c r="J63" s="12" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="9" t="n">
@@ -2505,15 +2295,12 @@
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr"/>
-      <c r="E64" s="11" t="inlineStr"/>
-      <c r="F64" s="11" t="inlineStr"/>
+      <c r="E64" s="12" t="inlineStr"/>
+      <c r="F64" s="12" t="inlineStr"/>
       <c r="G64" s="11" t="inlineStr"/>
       <c r="H64" s="11" t="inlineStr"/>
       <c r="I64" s="11" t="inlineStr"/>
-      <c r="J64" s="11" t="inlineStr"/>
-      <c r="K64" s="11" t="inlineStr"/>
-      <c r="L64" s="11" t="inlineStr"/>
-      <c r="M64" s="12" t="inlineStr"/>
+      <c r="J64" s="12" t="inlineStr"/>
     </row>
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="8" t="inlineStr">
@@ -2537,15 +2324,12 @@
         </is>
       </c>
       <c r="D66" s="11" t="inlineStr"/>
-      <c r="E66" s="11" t="inlineStr"/>
-      <c r="F66" s="11" t="inlineStr"/>
+      <c r="E66" s="12" t="inlineStr"/>
+      <c r="F66" s="12" t="inlineStr"/>
       <c r="G66" s="11" t="inlineStr"/>
       <c r="H66" s="11" t="inlineStr"/>
       <c r="I66" s="11" t="inlineStr"/>
-      <c r="J66" s="11" t="inlineStr"/>
-      <c r="K66" s="11" t="inlineStr"/>
-      <c r="L66" s="11" t="inlineStr"/>
-      <c r="M66" s="12" t="inlineStr"/>
+      <c r="J66" s="12" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="9" t="n">
@@ -2562,15 +2346,12 @@
         </is>
       </c>
       <c r="D67" s="11" t="inlineStr"/>
-      <c r="E67" s="11" t="inlineStr"/>
-      <c r="F67" s="11" t="inlineStr"/>
+      <c r="E67" s="12" t="inlineStr"/>
+      <c r="F67" s="12" t="inlineStr"/>
       <c r="G67" s="11" t="inlineStr"/>
       <c r="H67" s="11" t="inlineStr"/>
       <c r="I67" s="11" t="inlineStr"/>
-      <c r="J67" s="11" t="inlineStr"/>
-      <c r="K67" s="11" t="inlineStr"/>
-      <c r="L67" s="11" t="inlineStr"/>
-      <c r="M67" s="12" t="inlineStr"/>
+      <c r="J67" s="12" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="9" t="n">
@@ -2587,15 +2368,12 @@
         </is>
       </c>
       <c r="D68" s="11" t="inlineStr"/>
-      <c r="E68" s="11" t="inlineStr"/>
-      <c r="F68" s="11" t="inlineStr"/>
+      <c r="E68" s="12" t="inlineStr"/>
+      <c r="F68" s="12" t="inlineStr"/>
       <c r="G68" s="11" t="inlineStr"/>
       <c r="H68" s="11" t="inlineStr"/>
       <c r="I68" s="11" t="inlineStr"/>
-      <c r="J68" s="11" t="inlineStr"/>
-      <c r="K68" s="11" t="inlineStr"/>
-      <c r="L68" s="11" t="inlineStr"/>
-      <c r="M68" s="12" t="inlineStr"/>
+      <c r="J68" s="12" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="9" t="n">
@@ -2612,15 +2390,12 @@
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr"/>
-      <c r="E69" s="11" t="inlineStr"/>
-      <c r="F69" s="11" t="inlineStr"/>
+      <c r="E69" s="12" t="inlineStr"/>
+      <c r="F69" s="12" t="inlineStr"/>
       <c r="G69" s="11" t="inlineStr"/>
       <c r="H69" s="11" t="inlineStr"/>
       <c r="I69" s="11" t="inlineStr"/>
-      <c r="J69" s="11" t="inlineStr"/>
-      <c r="K69" s="11" t="inlineStr"/>
-      <c r="L69" s="11" t="inlineStr"/>
-      <c r="M69" s="12" t="inlineStr"/>
+      <c r="J69" s="12" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="9" t="n">
@@ -2637,15 +2412,12 @@
         </is>
       </c>
       <c r="D70" s="11" t="inlineStr"/>
-      <c r="E70" s="11" t="inlineStr"/>
-      <c r="F70" s="11" t="inlineStr"/>
+      <c r="E70" s="12" t="inlineStr"/>
+      <c r="F70" s="12" t="inlineStr"/>
       <c r="G70" s="11" t="inlineStr"/>
       <c r="H70" s="11" t="inlineStr"/>
       <c r="I70" s="11" t="inlineStr"/>
-      <c r="J70" s="11" t="inlineStr"/>
-      <c r="K70" s="11" t="inlineStr"/>
-      <c r="L70" s="11" t="inlineStr"/>
-      <c r="M70" s="12" t="inlineStr"/>
+      <c r="J70" s="12" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="9" t="n">
@@ -2662,15 +2434,12 @@
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr"/>
-      <c r="E71" s="11" t="inlineStr"/>
-      <c r="F71" s="11" t="inlineStr"/>
+      <c r="E71" s="12" t="inlineStr"/>
+      <c r="F71" s="12" t="inlineStr"/>
       <c r="G71" s="11" t="inlineStr"/>
       <c r="H71" s="11" t="inlineStr"/>
       <c r="I71" s="11" t="inlineStr"/>
-      <c r="J71" s="11" t="inlineStr"/>
-      <c r="K71" s="11" t="inlineStr"/>
-      <c r="L71" s="11" t="inlineStr"/>
-      <c r="M71" s="12" t="inlineStr"/>
+      <c r="J71" s="12" t="inlineStr"/>
     </row>
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="8" t="inlineStr">
@@ -2694,15 +2463,12 @@
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr"/>
-      <c r="E73" s="11" t="inlineStr"/>
-      <c r="F73" s="11" t="inlineStr"/>
+      <c r="E73" s="12" t="inlineStr"/>
+      <c r="F73" s="12" t="inlineStr"/>
       <c r="G73" s="11" t="inlineStr"/>
       <c r="H73" s="11" t="inlineStr"/>
       <c r="I73" s="11" t="inlineStr"/>
-      <c r="J73" s="11" t="inlineStr"/>
-      <c r="K73" s="11" t="inlineStr"/>
-      <c r="L73" s="11" t="inlineStr"/>
-      <c r="M73" s="12" t="inlineStr"/>
+      <c r="J73" s="12" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="n">
@@ -2719,15 +2485,12 @@
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr"/>
-      <c r="E74" s="11" t="inlineStr"/>
-      <c r="F74" s="11" t="inlineStr"/>
+      <c r="E74" s="12" t="inlineStr"/>
+      <c r="F74" s="12" t="inlineStr"/>
       <c r="G74" s="11" t="inlineStr"/>
       <c r="H74" s="11" t="inlineStr"/>
       <c r="I74" s="11" t="inlineStr"/>
-      <c r="J74" s="11" t="inlineStr"/>
-      <c r="K74" s="11" t="inlineStr"/>
-      <c r="L74" s="11" t="inlineStr"/>
-      <c r="M74" s="12" t="inlineStr"/>
+      <c r="J74" s="12" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="9" t="n">
@@ -2744,15 +2507,12 @@
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr"/>
-      <c r="E75" s="11" t="inlineStr"/>
-      <c r="F75" s="11" t="inlineStr"/>
+      <c r="E75" s="12" t="inlineStr"/>
+      <c r="F75" s="12" t="inlineStr"/>
       <c r="G75" s="11" t="inlineStr"/>
       <c r="H75" s="11" t="inlineStr"/>
       <c r="I75" s="11" t="inlineStr"/>
-      <c r="J75" s="11" t="inlineStr"/>
-      <c r="K75" s="11" t="inlineStr"/>
-      <c r="L75" s="11" t="inlineStr"/>
-      <c r="M75" s="12" t="inlineStr"/>
+      <c r="J75" s="12" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="9" t="n">
@@ -2769,15 +2529,12 @@
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr"/>
-      <c r="E76" s="11" t="inlineStr"/>
-      <c r="F76" s="11" t="inlineStr"/>
+      <c r="E76" s="12" t="inlineStr"/>
+      <c r="F76" s="12" t="inlineStr"/>
       <c r="G76" s="11" t="inlineStr"/>
       <c r="H76" s="11" t="inlineStr"/>
       <c r="I76" s="11" t="inlineStr"/>
-      <c r="J76" s="11" t="inlineStr"/>
-      <c r="K76" s="11" t="inlineStr"/>
-      <c r="L76" s="11" t="inlineStr"/>
-      <c r="M76" s="12" t="inlineStr"/>
+      <c r="J76" s="12" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="9" t="n">
@@ -2794,15 +2551,12 @@
         </is>
       </c>
       <c r="D77" s="11" t="inlineStr"/>
-      <c r="E77" s="11" t="inlineStr"/>
-      <c r="F77" s="11" t="inlineStr"/>
+      <c r="E77" s="12" t="inlineStr"/>
+      <c r="F77" s="12" t="inlineStr"/>
       <c r="G77" s="11" t="inlineStr"/>
       <c r="H77" s="11" t="inlineStr"/>
       <c r="I77" s="11" t="inlineStr"/>
-      <c r="J77" s="11" t="inlineStr"/>
-      <c r="K77" s="11" t="inlineStr"/>
-      <c r="L77" s="11" t="inlineStr"/>
-      <c r="M77" s="12" t="inlineStr"/>
+      <c r="J77" s="12" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="9" t="n">
@@ -2819,15 +2573,12 @@
         </is>
       </c>
       <c r="D78" s="11" t="inlineStr"/>
-      <c r="E78" s="11" t="inlineStr"/>
-      <c r="F78" s="11" t="inlineStr"/>
+      <c r="E78" s="12" t="inlineStr"/>
+      <c r="F78" s="12" t="inlineStr"/>
       <c r="G78" s="11" t="inlineStr"/>
       <c r="H78" s="11" t="inlineStr"/>
       <c r="I78" s="11" t="inlineStr"/>
-      <c r="J78" s="11" t="inlineStr"/>
-      <c r="K78" s="11" t="inlineStr"/>
-      <c r="L78" s="11" t="inlineStr"/>
-      <c r="M78" s="12" t="inlineStr"/>
+      <c r="J78" s="12" t="inlineStr"/>
     </row>
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="8" t="inlineStr">
@@ -2851,15 +2602,12 @@
         </is>
       </c>
       <c r="D80" s="11" t="inlineStr"/>
-      <c r="E80" s="11" t="inlineStr"/>
-      <c r="F80" s="11" t="inlineStr"/>
+      <c r="E80" s="12" t="inlineStr"/>
+      <c r="F80" s="12" t="inlineStr"/>
       <c r="G80" s="11" t="inlineStr"/>
       <c r="H80" s="11" t="inlineStr"/>
       <c r="I80" s="11" t="inlineStr"/>
-      <c r="J80" s="11" t="inlineStr"/>
-      <c r="K80" s="11" t="inlineStr"/>
-      <c r="L80" s="11" t="inlineStr"/>
-      <c r="M80" s="12" t="inlineStr"/>
+      <c r="J80" s="12" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="9" t="n">
@@ -2876,15 +2624,12 @@
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr"/>
-      <c r="E81" s="11" t="inlineStr"/>
-      <c r="F81" s="11" t="inlineStr"/>
+      <c r="E81" s="12" t="inlineStr"/>
+      <c r="F81" s="12" t="inlineStr"/>
       <c r="G81" s="11" t="inlineStr"/>
       <c r="H81" s="11" t="inlineStr"/>
       <c r="I81" s="11" t="inlineStr"/>
-      <c r="J81" s="11" t="inlineStr"/>
-      <c r="K81" s="11" t="inlineStr"/>
-      <c r="L81" s="11" t="inlineStr"/>
-      <c r="M81" s="12" t="inlineStr"/>
+      <c r="J81" s="12" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="9" t="n">
@@ -2901,15 +2646,12 @@
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr"/>
-      <c r="E82" s="11" t="inlineStr"/>
-      <c r="F82" s="11" t="inlineStr"/>
+      <c r="E82" s="12" t="inlineStr"/>
+      <c r="F82" s="12" t="inlineStr"/>
       <c r="G82" s="11" t="inlineStr"/>
       <c r="H82" s="11" t="inlineStr"/>
       <c r="I82" s="11" t="inlineStr"/>
-      <c r="J82" s="11" t="inlineStr"/>
-      <c r="K82" s="11" t="inlineStr"/>
-      <c r="L82" s="11" t="inlineStr"/>
-      <c r="M82" s="12" t="inlineStr"/>
+      <c r="J82" s="12" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="9" t="n">
@@ -2926,15 +2668,12 @@
         </is>
       </c>
       <c r="D83" s="11" t="inlineStr"/>
-      <c r="E83" s="11" t="inlineStr"/>
-      <c r="F83" s="11" t="inlineStr"/>
+      <c r="E83" s="12" t="inlineStr"/>
+      <c r="F83" s="12" t="inlineStr"/>
       <c r="G83" s="11" t="inlineStr"/>
       <c r="H83" s="11" t="inlineStr"/>
       <c r="I83" s="11" t="inlineStr"/>
-      <c r="J83" s="11" t="inlineStr"/>
-      <c r="K83" s="11" t="inlineStr"/>
-      <c r="L83" s="11" t="inlineStr"/>
-      <c r="M83" s="12" t="inlineStr"/>
+      <c r="J83" s="12" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="9" t="n">
@@ -2951,15 +2690,12 @@
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr"/>
-      <c r="E84" s="11" t="inlineStr"/>
-      <c r="F84" s="11" t="inlineStr"/>
+      <c r="E84" s="12" t="inlineStr"/>
+      <c r="F84" s="12" t="inlineStr"/>
       <c r="G84" s="11" t="inlineStr"/>
       <c r="H84" s="11" t="inlineStr"/>
       <c r="I84" s="11" t="inlineStr"/>
-      <c r="J84" s="11" t="inlineStr"/>
-      <c r="K84" s="11" t="inlineStr"/>
-      <c r="L84" s="11" t="inlineStr"/>
-      <c r="M84" s="12" t="inlineStr"/>
+      <c r="J84" s="12" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="9" t="n">
@@ -2976,32 +2712,29 @@
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr"/>
-      <c r="E85" s="11" t="inlineStr"/>
-      <c r="F85" s="11" t="inlineStr"/>
+      <c r="E85" s="12" t="inlineStr"/>
+      <c r="F85" s="12" t="inlineStr"/>
       <c r="G85" s="11" t="inlineStr"/>
       <c r="H85" s="11" t="inlineStr"/>
       <c r="I85" s="11" t="inlineStr"/>
-      <c r="J85" s="11" t="inlineStr"/>
-      <c r="K85" s="11" t="inlineStr"/>
-      <c r="L85" s="11" t="inlineStr"/>
-      <c r="M85" s="12" t="inlineStr"/>
+      <c r="J85" s="12" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A44:M44"/>
-    <mergeCell ref="A23:M23"/>
-    <mergeCell ref="A37:M37"/>
-    <mergeCell ref="A79:M79"/>
-    <mergeCell ref="A58:M58"/>
-    <mergeCell ref="A9:M9"/>
-    <mergeCell ref="A30:M30"/>
-    <mergeCell ref="A72:M72"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A65:M65"/>
-    <mergeCell ref="A16:M16"/>
-    <mergeCell ref="A51:M51"/>
+    <mergeCell ref="A44:J44"/>
+    <mergeCell ref="A23:J23"/>
+    <mergeCell ref="A37:J37"/>
+    <mergeCell ref="A79:J79"/>
+    <mergeCell ref="A58:J58"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A30:J30"/>
+    <mergeCell ref="A65:J65"/>
+    <mergeCell ref="A16:J16"/>
+    <mergeCell ref="A72:J72"/>
+    <mergeCell ref="A51:J51"/>
   </mergeCells>
-  <conditionalFormatting sqref="J2:J85">
+  <conditionalFormatting sqref="I2:I85">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"At risk"</formula>
     </cfRule>
@@ -3012,21 +2745,15 @@
       <formula>"On track"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="5">
+  <dataValidations count="3">
     <dataValidation sqref="D2:D85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,Excused"</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Up,Flat,Down"</formula1>
+      <formula1>"0,1,2,3,4,5,6,7,8,9,10"</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Positive,Neutral,Low"</formula1>
-    </dataValidation>
-    <dataValidation sqref="J2:J85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"On track,Watch,At risk"</formula1>
-    </dataValidation>
-    <dataValidation sqref="L2:L85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3039,7 +2766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X19"/>
+  <dimension ref="A1:Y19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3066,6 +2793,7 @@
     <col width="10" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
     <col width="52" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -3189,6 +2917,11 @@
           <t>Mentor notes / next steps</t>
         </is>
       </c>
+      <c r="Y1" s="7" t="inlineStr">
+        <is>
+          <t>Points to date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -3293,6 +3026,10 @@
           <t>Two submissions waiting. JWT refresh-token blocker flagged early. Pair on auth Thursday.</t>
         </is>
       </c>
+      <c r="Y2" s="13">
+        <f>IF(B2="","",SUMIF('Weekly Tracker'!$C:$C,B2,'Weekly Tracker'!$H:$H))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -3397,6 +3134,10 @@
           <t>Power outages and a shared machine. Struggling despite effort. Protect deadlines, shift due times to AM PKT.</t>
         </is>
       </c>
+      <c r="Y3" s="13">
+        <f>IF(B3="","",SUMIF('Weekly Tracker'!$C:$C,B3,'Weekly Tracker'!$H:$H))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -3501,6 +3242,10 @@
           <t>Disengagement risk. No login for 6 days, two nudges unanswered. Direct warm check-in. Psychologist session held May 20.</t>
         </is>
       </c>
+      <c r="Y4" s="13">
+        <f>IF(B4="","",SUMIF('Weekly Tracker'!$C:$C,B4,'Weekly Tracker'!$H:$H))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -3605,6 +3350,10 @@
           <t>Top of cohort on output, almost always early. May be coasting on easy ground. Add a stretch track.</t>
         </is>
       </c>
+      <c r="Y5" s="13">
+        <f>IF(B5="","",SUMIF('Weekly Tracker'!$C:$C,B5,'Weekly Tracker'!$H:$H))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -3709,6 +3458,10 @@
           <t>Solid and improving three weeks running. One async/await blocker, working at it.</t>
         </is>
       </c>
+      <c r="Y6" s="13">
+        <f>IF(B6="","",SUMIF('Weekly Tracker'!$C:$C,B6,'Weekly Tracker'!$H:$H))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -3812,6 +3565,10 @@
         <is>
           <t>Drifting, two late tasks this week. Still responsive. A short check-in now prevents a bigger slide.</t>
         </is>
+      </c>
+      <c r="Y7" s="13">
+        <f>IF(B7="","",SUMIF('Weekly Tracker'!$C:$C,B7,'Weekly Tracker'!$H:$H))</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -3839,6 +3596,10 @@
       <c r="V8" s="11" t="inlineStr"/>
       <c r="W8" s="11" t="inlineStr"/>
       <c r="X8" s="12" t="inlineStr"/>
+      <c r="Y8" s="13">
+        <f>IF(B8="","",SUMIF('Weekly Tracker'!$C:$C,B8,'Weekly Tracker'!$H:$H))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr"/>
@@ -3865,6 +3626,10 @@
       <c r="V9" s="11" t="inlineStr"/>
       <c r="W9" s="11" t="inlineStr"/>
       <c r="X9" s="12" t="inlineStr"/>
+      <c r="Y9" s="13">
+        <f>IF(B9="","",SUMIF('Weekly Tracker'!$C:$C,B9,'Weekly Tracker'!$H:$H))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr"/>
@@ -3891,6 +3656,10 @@
       <c r="V10" s="11" t="inlineStr"/>
       <c r="W10" s="11" t="inlineStr"/>
       <c r="X10" s="12" t="inlineStr"/>
+      <c r="Y10" s="13">
+        <f>IF(B10="","",SUMIF('Weekly Tracker'!$C:$C,B10,'Weekly Tracker'!$H:$H))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr"/>
@@ -3917,6 +3686,10 @@
       <c r="V11" s="11" t="inlineStr"/>
       <c r="W11" s="11" t="inlineStr"/>
       <c r="X11" s="12" t="inlineStr"/>
+      <c r="Y11" s="13">
+        <f>IF(B11="","",SUMIF('Weekly Tracker'!$C:$C,B11,'Weekly Tracker'!$H:$H))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr"/>
@@ -3943,6 +3716,10 @@
       <c r="V12" s="11" t="inlineStr"/>
       <c r="W12" s="11" t="inlineStr"/>
       <c r="X12" s="12" t="inlineStr"/>
+      <c r="Y12" s="13">
+        <f>IF(B12="","",SUMIF('Weekly Tracker'!$C:$C,B12,'Weekly Tracker'!$H:$H))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr"/>
@@ -3969,6 +3746,10 @@
       <c r="V13" s="11" t="inlineStr"/>
       <c r="W13" s="11" t="inlineStr"/>
       <c r="X13" s="12" t="inlineStr"/>
+      <c r="Y13" s="13">
+        <f>IF(B13="","",SUMIF('Weekly Tracker'!$C:$C,B13,'Weekly Tracker'!$H:$H))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr"/>
@@ -3995,6 +3776,10 @@
       <c r="V14" s="11" t="inlineStr"/>
       <c r="W14" s="11" t="inlineStr"/>
       <c r="X14" s="12" t="inlineStr"/>
+      <c r="Y14" s="13">
+        <f>IF(B14="","",SUMIF('Weekly Tracker'!$C:$C,B14,'Weekly Tracker'!$H:$H))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr"/>
@@ -4021,6 +3806,10 @@
       <c r="V15" s="11" t="inlineStr"/>
       <c r="W15" s="11" t="inlineStr"/>
       <c r="X15" s="12" t="inlineStr"/>
+      <c r="Y15" s="13">
+        <f>IF(B15="","",SUMIF('Weekly Tracker'!$C:$C,B15,'Weekly Tracker'!$H:$H))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr"/>
@@ -4047,6 +3836,10 @@
       <c r="V16" s="11" t="inlineStr"/>
       <c r="W16" s="11" t="inlineStr"/>
       <c r="X16" s="12" t="inlineStr"/>
+      <c r="Y16" s="13">
+        <f>IF(B16="","",SUMIF('Weekly Tracker'!$C:$C,B16,'Weekly Tracker'!$H:$H))</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr"/>
@@ -4073,6 +3866,10 @@
       <c r="V17" s="11" t="inlineStr"/>
       <c r="W17" s="11" t="inlineStr"/>
       <c r="X17" s="12" t="inlineStr"/>
+      <c r="Y17" s="13">
+        <f>IF(B17="","",SUMIF('Weekly Tracker'!$C:$C,B17,'Weekly Tracker'!$H:$H))</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr"/>
@@ -4099,6 +3896,10 @@
       <c r="V18" s="11" t="inlineStr"/>
       <c r="W18" s="11" t="inlineStr"/>
       <c r="X18" s="12" t="inlineStr"/>
+      <c r="Y18" s="13">
+        <f>IF(B18="","",SUMIF('Weekly Tracker'!$C:$C,B18,'Weekly Tracker'!$H:$H))</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr"/>
@@ -4125,6 +3926,10 @@
       <c r="V19" s="11" t="inlineStr"/>
       <c r="W19" s="11" t="inlineStr"/>
       <c r="X19" s="12" t="inlineStr"/>
+      <c r="Y19" s="13">
+        <f>IF(B19="","",SUMIF('Weekly Tracker'!$C:$C,B19,'Weekly Tracker'!$H:$H))</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="N2:N19">

</xml_diff>